<commit_message>
Add text for introductory validate example
</commit_message>
<xml_diff>
--- a/data/dog_walks.xlsx
+++ b/data/dog_walks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scotsconnect.sharepoint.com/sites/msteams_ab71a5_342727/Shared Documents/data_validation_intro_training/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33534BDF-85F4-4880-A259-EFED4A6624DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{C193DD5A-FF16-43E7-8BBB-414C0F65B118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{166C9BCA-2C49-4C94-B9D7-16ED7B1B34D6}"/>
   <bookViews>
     <workbookView xWindow="165" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{97492233-ED57-4AE6-B24C-B307BD121A43}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="27">
   <si>
     <t>dog_name</t>
   </si>
@@ -71,18 +71,12 @@
     <t>Milo</t>
   </si>
   <si>
-    <t>Rocky</t>
-  </si>
-  <si>
     <t>Coco</t>
   </si>
   <si>
     <t>Buddy</t>
   </si>
   <si>
-    <t>dog_breed</t>
-  </si>
-  <si>
     <t>Labrador</t>
   </si>
   <si>
@@ -116,13 +110,13 @@
     <t>unknown</t>
   </si>
   <si>
-    <t>energy_after</t>
-  </si>
-  <si>
     <t>date_of_walk</t>
   </si>
   <si>
     <t>walk_id</t>
+  </si>
+  <si>
+    <t>dog_bread</t>
   </si>
 </sst>
 </file>
@@ -495,7 +489,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2F9ED11-8D2B-4E41-A6FA-C4E674309E6C}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
@@ -506,24 +500,23 @@
     <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
@@ -534,11 +527,8 @@
       <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -546,10 +536,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E2" s="1">
         <v>46132</v>
@@ -563,11 +553,8 @@
       <c r="H2">
         <v>5</v>
       </c>
-      <c r="I2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -575,10 +562,10 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1">
         <v>46132</v>
@@ -592,11 +579,8 @@
       <c r="H3">
         <v>2</v>
       </c>
-      <c r="I3">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -604,10 +588,10 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1">
         <v>46132</v>
@@ -621,11 +605,8 @@
       <c r="H4">
         <v>12</v>
       </c>
-      <c r="I4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -633,10 +614,10 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E5" s="1">
         <v>46132</v>
@@ -650,11 +631,8 @@
       <c r="H5">
         <v>3</v>
       </c>
-      <c r="I5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -662,10 +640,10 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E6" s="1">
         <v>46133</v>
@@ -679,11 +657,8 @@
       <c r="H6">
         <v>1</v>
       </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -691,10 +666,10 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="E7" s="1">
         <v>46133</v>
@@ -705,11 +680,8 @@
       <c r="H7">
         <v>4</v>
       </c>
-      <c r="I7">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -717,10 +689,10 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1">
         <v>46133</v>
@@ -734,22 +706,19 @@
       <c r="H8">
         <v>999</v>
       </c>
-      <c r="I8">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>11</v>
+      <c r="B9">
+        <v>123</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E9" s="1">
         <v>46133</v>
@@ -763,22 +732,16 @@
       <c r="H9">
         <v>6</v>
       </c>
-      <c r="I9">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E10" s="1">
         <v>46134</v>
@@ -792,22 +755,19 @@
       <c r="H10">
         <v>2</v>
       </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
         <v>13</v>
       </c>
-      <c r="C11" t="s">
-        <v>15</v>
-      </c>
       <c r="D11" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E11" s="1">
         <v>46134</v>
@@ -818,11 +778,8 @@
       <c r="G11">
         <v>60</v>
       </c>
-      <c r="I11">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -830,10 +787,10 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E12" s="1">
         <v>46134</v>
@@ -847,22 +804,19 @@
       <c r="H12">
         <v>4</v>
       </c>
-      <c r="I12">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E13" s="1">
         <v>46134</v>
@@ -875,9 +829,6 @@
       </c>
       <c r="H13">
         <v>2</v>
-      </c>
-      <c r="I13">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1129,13 +1080,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C296622-5F2D-4E3C-BAA9-53E7825871F6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C296622-5F2D-4E3C-BAA9-53E7825871F6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d6e8461a-a6a2-4e4e-936d-1d1c7577dac5"/>
+    <ds:schemaRef ds:uri="169a8418-a667-4c9d-8dbd-7e109047e3ad"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4899F08E-38BB-4AD8-A81C-89128CECBDED}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4899F08E-38BB-4AD8-A81C-89128CECBDED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BAC2A0D-B2BF-4787-9C14-CBAF2430F82F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BAC2A0D-B2BF-4787-9C14-CBAF2430F82F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="169a8418-a667-4c9d-8dbd-7e109047e3ad"/>
+    <ds:schemaRef ds:uri="d6e8461a-a6a2-4e4e-936d-1d1c7577dac5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>